<commit_message>
old version 77 added
</commit_message>
<xml_diff>
--- a/meal sucrose drink.xlsx
+++ b/meal sucrose drink.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBD9D14-AB48-4247-A21A-98D880138947}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{3BBD9D14-AB48-4247-A21A-98D880138947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59A187FC-D740-4360-8DE5-F1198377AC3E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -500,7 +505,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -516,7 +521,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="meal"/>
@@ -644,10 +649,14 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -685,9 +694,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -720,26 +729,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -772,26 +764,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1053,7 +1028,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="9">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C6" s="7">
         <v>250</v>

</xml_diff>